<commit_message>
Feat(DarkMode): ajout d'un dark mode
[20][WPI]
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3636,7 +3636,6 @@
 
 <file path=xl/charts/chart37.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3781,6 +3780,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -3796,6 +3803,119 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart39.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -3900,6 +4020,117 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart40.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -5389,6 +5620,50 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="39" name="Chart 39"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId39"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="40" name="Chart 40"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId40"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -5681,7 +5956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5962,57 +6237,156 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Chor(Save): Save code on cloud</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>[1]</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>[TEST]</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Chor(Save): Save code on cloud</t>
-        </is>
-      </c>
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>2h15 (135 min)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2h16 (136 min)</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>FIX(Get_commit): ca ne fonctionnais pas chez mes camarades</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>il avait modif les dates et il ne faut surtout pas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Fix(Reload): Reload infini</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>[6]</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Fix(Reload): Reload infini</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Feat(detail): affiche les detail d'un livre avec le bouton pour lire</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>[15]</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Feat(detail): affiche les detail d'un livre avec le bouton pour lire</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Feat(Résumé): Ouvre le pdf de résumer</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Feat(Résumé): Ouvre le pdf de résumer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>1h11 (71 min)</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
-  <mergeCells count="4">
+  <autoFilter ref="A1:E23"/>
+  <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6098,7 +6472,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -6116,14 +6490,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>2.27</v>
+        <v>2.25</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2h16</t>
+          <t>2h15</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -6133,7 +6507,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4h07</t>
+          <t>5h17</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6142,10 +6516,26 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>4.12</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>71</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1h11</t>
+        </is>
+      </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Moyenne / jour</t>
@@ -6153,8 +6543,16 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h04</t>
-        </is>
+          <t>1h46</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>5.28</v>
       </c>
     </row>
     <row r="5">
@@ -6165,12 +6563,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>25/03/2026 (2h16)</t>
+          <t>25/03/2026 (2h15)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Feat(nouvelle api): Api de Théo
[1h30][DONE]
Je n'arrive a pas grand chose pour le moment. ca run mais je n'arrive a
rien avec les epub
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -4448,7 +4448,6 @@
 
 <file path=xl/charts/chart43.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4593,6 +4592,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -4608,6 +4615,580 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart45.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart46.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart47.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart48.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart49.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -4782,6 +5363,1161 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart50.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart51.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart52.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart53.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart54.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart55.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart56.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart57.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart58.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart59.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -4824,6 +6560,580 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart60.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart61.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart62.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart63.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart64.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -6214,6 +8524,446 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="45" name="Chart 45"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId45"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="46" name="Chart 46"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId46"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="47" name="Chart 47"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId47"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="48" name="Chart 48"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId48"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="49" name="Chart 49"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId49"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="50" name="Chart 50"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId50"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="51" name="Chart 51"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId51"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="52" name="Chart 52"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId52"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="53" name="Chart 53"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId53"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="54" name="Chart 54"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId54"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="55" name="Chart 55"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId55"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="56" name="Chart 56"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId56"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="57" name="Chart 57"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId57"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="58" name="Chart 58"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId58"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="59" name="Chart 59"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId59"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="60" name="Chart 60"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId60"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="61" name="Chart 61"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId61"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="62" name="Chart 62"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId62"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="63" name="Chart 63"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId63"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="64" name="Chart 64"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId64"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -6957,12 +9707,12 @@
       <c r="A24" s="3" t="inlineStr"/>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Sauvegarde</t>
+          <t>Chor(JNR)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[0]</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6972,7 +9722,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Sauvegarde du code sur le cloud</t>
+          <t>Chor(JNR)</t>
         </is>
       </c>
     </row>
@@ -6985,7 +9735,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>2h15 (135 min)</t>
+          <t>2h11 (131 min)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -7126,7 +9876,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6h21</t>
+          <t>6h17</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7145,14 +9895,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C4" t="n">
-        <v>2.25</v>
+        <v>2.18</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2h15</t>
+          <t>2h11</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -7162,7 +9912,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h07</t>
+          <t>2h06</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7171,7 +9921,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>6.35</v>
+        <v>6.28</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
chore: update journal de travail
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6989,7 +6989,6 @@
 
 <file path=xl/charts/chart63.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -7134,6 +7133,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -7142,6 +7149,230 @@
           <val>
             <numRef>
               <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart65.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart66.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
             </numRef>
           </val>
         </ser>
@@ -8964,6 +9195,50 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="65" name="Chart 65"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId65"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="66" name="Chart 66"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId66"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -9256,7 +9531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9748,14 +10023,288 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Feat(nouvelle api): Api de Théo</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>[1h30]</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Feat(nouvelle api): Api de Théo  Je n'arrive a pas grand chose pour le moment. ca run mais je n'arrive a rien avec les epub</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Feat(api): tentative de epub</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>[1h30]</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Feat(api): tentative de epub  ca marche pas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>3h00 (180 min)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Fix(loading): lazy loading + UI improvements</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Fix(loading): lazy loading + UI improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Feat(API): api custom</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Feat(API): api custom</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0h50 (50 min)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Feat: add custom api for mobile</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Feat: add custom api for mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr"/>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Feat: add more input on add page</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>[13]</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Feat: add more input on add page</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>feat: sqlight</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>[60]</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>feat: sqlight</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr"/>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Feat: epub</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>[7]</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Feat: epub</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>2h00 (120 min)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
-  <mergeCells count="5">
+  <autoFilter ref="A1:E43"/>
+  <mergeCells count="8">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9767,7 +10316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9841,7 +10390,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -9876,7 +10425,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6h17</t>
+          <t>12h07</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -9912,7 +10461,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h06</t>
+          <t>2h01</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -9925,6 +10474,22 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>180</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3h00</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Jour le plus charge</t>
@@ -9932,12 +10497,72 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>25/03/2026 (2h15)</t>
-        </is>
+          <t>22/04/2026 (3h00)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>9.279999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0h50</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>10.12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>120</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2h00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>12.12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D4"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
doc: readme et teste d' Tests fonctionnels
[30][DONE]
le readme decris comment lancer l'api et l'app. Les tests fonctionnels
sont également dans le readme
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -3,15 +3,15 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$F$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$9</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,13 +20,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -56,7 +62,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +85,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEEF5FC"/>
         <bgColor rgb="FFEEF5FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF455A64"/>
+        <bgColor rgb="FF455A64"/>
       </patternFill>
     </fill>
     <fill>
@@ -109,6 +121,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF6A1B9A"/>
         <bgColor rgb="FF6A1B9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4527A0"/>
+        <bgColor rgb="FF4527A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
@@ -161,14 +185,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="004527A0"/>
+        <bgColor rgb="004527A0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004527A0"/>
-        <bgColor rgb="004527A0"/>
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -184,59 +208,69 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,9 +395,9 @@
           <invertIfNegative val="1"/>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -381,16 +415,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -408,6 +448,12 @@
                 </pt>
                 <pt idx="5">
                   <v>2</v>
+                </pt>
+                <pt idx="6">
+                  <v>2.33</v>
+                </pt>
+                <pt idx="7">
+                  <v>0</v>
                 </pt>
               </numCache>
             </numRef>
@@ -511,7 +557,6 @@
       <tx>
         <rich>
           <a:bodyPr/>
-          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
@@ -522,25 +567,16 @@
           </a:p>
         </rich>
       </tx>
-      <overlay val="1"/>
     </title>
     <plotArea>
-      <layout/>
       <lineChart>
         <grouping val="standard"/>
-        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Tableau de bord'!$J$1</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Cumul (h)</v>
-                </pt>
-              </strCache>
+              <f>'Tableau de bord'!J1</f>
             </strRef>
           </tx>
           <spPr>
@@ -557,70 +593,17 @@
             </spPr>
           </marker>
           <cat>
-            <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>18/03/2026</v>
-                </pt>
-                <pt idx="1">
-                  <v>25/03/2026</v>
-                </pt>
-                <pt idx="2">
-                  <v>01/04/2026</v>
-                </pt>
-                <pt idx="3">
-                  <v>22/04/2026</v>
-                </pt>
-                <pt idx="4">
-                  <v>29/04/2026</v>
-                </pt>
-                <pt idx="5">
-                  <v>06/05/2026</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>1.85</v>
-                </pt>
-                <pt idx="1">
-                  <v>4.1</v>
-                </pt>
-                <pt idx="2">
-                  <v>6.28</v>
-                </pt>
-                <pt idx="3">
-                  <v>9.279999999999999</v>
-                </pt>
-                <pt idx="4">
-                  <v>10.12</v>
-                </pt>
-                <pt idx="5">
-                  <v>12.12</v>
-                </pt>
-              </numCache>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <marker val="1"/>
-        <smooth val="0"/>
+        <smooth val="1"/>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -629,13 +612,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -646,32 +627,23 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -682,20 +654,14 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -740,12 +706,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -859,12 +825,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
             </numRef>
           </val>
         </ser>
@@ -971,12 +937,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -1090,12 +1056,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
             </numRef>
           </val>
         </ser>
@@ -1167,6 +1133,7 @@
 
 <file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1202,12 +1169,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -1311,22 +1278,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
             </numRef>
           </val>
         </ser>
@@ -1334,350 +1293,6 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Charge par jour (heures)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Cumul des heures</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!J1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <smooth val="1"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Charge par jour (heures)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -1794,9 +1409,9 @@
           </marker>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -1814,16 +1429,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -1841,6 +1462,12 @@
                 </pt>
                 <pt idx="5">
                   <v>12.12</v>
+                </pt>
+                <pt idx="6">
+                  <v>14.45</v>
+                </pt>
+                <pt idx="7">
+                  <v>14.45</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1938,117 +1565,6 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Cumul des heures</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!J1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <smooth val="1"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -2097,9 +1613,9 @@
           <invertIfNegative val="1"/>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -2117,16 +1633,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -2144,6 +1666,12 @@
                 </pt>
                 <pt idx="5">
                   <v>2</v>
+                </pt>
+                <pt idx="6">
+                  <v>2.33</v>
+                </pt>
+                <pt idx="7">
+                  <v>0</v>
                 </pt>
               </numCache>
             </numRef>
@@ -2294,9 +1822,9 @@
           </marker>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -2314,16 +1842,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -2341,6 +1875,12 @@
                 </pt>
                 <pt idx="5">
                   <v>12.12</v>
+                </pt>
+                <pt idx="6">
+                  <v>14.45</v>
+                </pt>
+                <pt idx="7">
+                  <v>14.45</v>
                 </pt>
               </numCache>
             </numRef>
@@ -2486,9 +2026,9 @@
           <invertIfNegative val="1"/>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -2506,16 +2046,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -2533,6 +2079,12 @@
                 </pt>
                 <pt idx="5">
                   <v>2</v>
+                </pt>
+                <pt idx="6">
+                  <v>2.33</v>
+                </pt>
+                <pt idx="7">
+                  <v>0</v>
                 </pt>
               </numCache>
             </numRef>
@@ -2683,9 +2235,9 @@
           </marker>
           <cat>
             <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
               <strCache>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>18/03/2026</v>
                 </pt>
@@ -2703,16 +2255,22 @@
                 </pt>
                 <pt idx="5">
                   <v>06/05/2026</v>
+                </pt>
+                <pt idx="6">
+                  <v>13/05/2026</v>
+                </pt>
+                <pt idx="7">
+                  <v>20/05/2026</v>
                 </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
               <numCache>
                 <formatCode>General</formatCode>
-                <ptCount val="6"/>
+                <ptCount val="8"/>
                 <pt idx="0">
                   <v>1.85</v>
                 </pt>
@@ -2730,6 +2288,12 @@
                 </pt>
                 <pt idx="5">
                   <v>12.12</v>
+                </pt>
+                <pt idx="6">
+                  <v>14.45</v>
+                </pt>
+                <pt idx="7">
+                  <v>14.45</v>
                 </pt>
               </numCache>
             </numRef>
@@ -2744,6 +2308,7 @@
           <showPercent val="0"/>
           <showBubbleSize val="0"/>
         </dLbls>
+        <marker val="1"/>
         <smooth val="0"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -2834,7 +2399,6 @@
       <tx>
         <rich>
           <a:bodyPr/>
-          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
@@ -2845,26 +2409,17 @@
           </a:p>
         </rich>
       </tx>
-      <overlay val="1"/>
     </title>
     <plotArea>
-      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
-        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Tableau de bord'!$C$1</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Total (h)</v>
-                </pt>
-              </strCache>
+              <f>'Tableau de bord'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -2872,69 +2427,17 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <invertIfNegative val="1"/>
           <cat>
-            <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>18/03/2026</v>
-                </pt>
-                <pt idx="1">
-                  <v>25/03/2026</v>
-                </pt>
-                <pt idx="2">
-                  <v>01/04/2026</v>
-                </pt>
-                <pt idx="3">
-                  <v>22/04/2026</v>
-                </pt>
-                <pt idx="4">
-                  <v>29/04/2026</v>
-                </pt>
-                <pt idx="5">
-                  <v>06/05/2026</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>1.85</v>
-                </pt>
-                <pt idx="1">
-                  <v>2.25</v>
-                </pt>
-                <pt idx="2">
-                  <v>2.18</v>
-                </pt>
-                <pt idx="3">
-                  <v>3</v>
-                </pt>
-                <pt idx="4">
-                  <v>0.83</v>
-                </pt>
-                <pt idx="5">
-                  <v>2</v>
-                </pt>
-              </numCache>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -2944,13 +2447,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -2961,32 +2462,23 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -2997,20 +2489,14 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -3025,7 +2511,6 @@
       <tx>
         <rich>
           <a:bodyPr/>
-          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
@@ -3036,25 +2521,16 @@
           </a:p>
         </rich>
       </tx>
-      <overlay val="1"/>
     </title>
     <plotArea>
-      <layout/>
       <lineChart>
         <grouping val="standard"/>
-        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Tableau de bord'!$J$1</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Cumul (h)</v>
-                </pt>
-              </strCache>
+              <f>'Tableau de bord'!J1</f>
             </strRef>
           </tx>
           <spPr>
@@ -3071,69 +2547,17 @@
             </spPr>
           </marker>
           <cat>
-            <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>18/03/2026</v>
-                </pt>
-                <pt idx="1">
-                  <v>25/03/2026</v>
-                </pt>
-                <pt idx="2">
-                  <v>01/04/2026</v>
-                </pt>
-                <pt idx="3">
-                  <v>22/04/2026</v>
-                </pt>
-                <pt idx="4">
-                  <v>29/04/2026</v>
-                </pt>
-                <pt idx="5">
-                  <v>06/05/2026</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$7</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>1.85</v>
-                </pt>
-                <pt idx="1">
-                  <v>4.1</v>
-                </pt>
-                <pt idx="2">
-                  <v>6.28</v>
-                </pt>
-                <pt idx="3">
-                  <v>9.279999999999999</v>
-                </pt>
-                <pt idx="4">
-                  <v>10.12</v>
-                </pt>
-                <pt idx="5">
-                  <v>12.12</v>
-                </pt>
-              </numCache>
+              <f>'Tableau de bord'!$J$2:$J$9</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <smooth val="0"/>
+        <smooth val="1"/>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -3142,13 +2566,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -3159,32 +2581,23 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -3195,20 +2608,14 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -3223,7 +2630,6 @@
       <tx>
         <rich>
           <a:bodyPr/>
-          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
@@ -3234,26 +2640,17 @@
           </a:p>
         </rich>
       </tx>
-      <overlay val="1"/>
     </title>
     <plotArea>
-      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
-        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Tableau de bord'!$C$1</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Total (h)</v>
-                </pt>
-              </strCache>
+              <f>'Tableau de bord'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -3261,69 +2658,17 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <invertIfNegative val="1"/>
           <cat>
-            <strRef>
-              <f>'Tableau de bord'!$A$2:$A$7</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>18/03/2026</v>
-                </pt>
-                <pt idx="1">
-                  <v>25/03/2026</v>
-                </pt>
-                <pt idx="2">
-                  <v>01/04/2026</v>
-                </pt>
-                <pt idx="3">
-                  <v>22/04/2026</v>
-                </pt>
-                <pt idx="4">
-                  <v>29/04/2026</v>
-                </pt>
-                <pt idx="5">
-                  <v>06/05/2026</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$9</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$7</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>1.85</v>
-                </pt>
-                <pt idx="1">
-                  <v>2.25</v>
-                </pt>
-                <pt idx="2">
-                  <v>2.18</v>
-                </pt>
-                <pt idx="3">
-                  <v>3</v>
-                </pt>
-                <pt idx="4">
-                  <v>0.83</v>
-                </pt>
-                <pt idx="5">
-                  <v>2</v>
-                </pt>
-              </numCache>
+              <f>'Tableau de bord'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -3333,13 +2678,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -3350,32 +2693,23 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="1"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
           <tx>
             <rich>
               <a:bodyPr/>
-              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -3386,20 +2720,14 @@
               </a:p>
             </rich>
           </tx>
-          <overlay val="1"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -3761,94 +3089,6 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>7</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="17" name="Chart 17"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId17"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="18" name="Chart 18"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId18"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>7</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="19" name="Chart 19"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId19"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="20" name="Chart 20"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId20"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -4141,15 +3381,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="11" min="1" max="1"/>
-    <col width="18" customWidth="1" style="11" min="2" max="2"/>
-    <col width="45" customWidth="1" style="11" min="3" max="3"/>
-    <col width="14" customWidth="1" style="11" min="4" max="4"/>
-    <col width="10" customWidth="1" style="11" min="5" max="5"/>
-    <col width="80" customWidth="1" style="11" min="6" max="6"/>
+    <col width="14" customWidth="1" style="15" min="1" max="1"/>
+    <col width="18" customWidth="1" style="15" min="2" max="2"/>
+    <col width="75" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
+    <col width="16" customWidth="1" style="15" min="4" max="4"/>
+    <col width="12" customWidth="1" style="15" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4165,7 +3404,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Nom</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -4178,106 +3417,85 @@
           <t>État</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>18/03/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr"/>
-      <c r="B3" s="14" t="inlineStr"/>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Maquette</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr"/>
+      <c r="B3" s="18" t="inlineStr"/>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Conception et réalisation de la maquette de l'interface utilisateur de l'application.</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>[55]</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>Maquette de l'application</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr"/>
-      <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>Creation de Get_commit</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr"/>
+      <c r="B4" s="18" t="inlineStr"/>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Création et configuration du script automatisé Get_commit.sh afin de récupérer les commits Git pour alimenter le journal de travail.</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>[55]</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Creation du script Get_commit.sh pour récupérer les commits pour faire le journal de travail</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr"/>
-      <c r="B5" s="14" t="inlineStr"/>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Initial commit</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr"/>
+      <c r="B5" s="18" t="inlineStr"/>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Initialisation du dépôt Git du projet.</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>[1]</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Initial commit</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr"/>
-      <c r="B6" s="15" t="inlineStr"/>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr"/>
+      <c r="B6" s="19" t="inlineStr"/>
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>1h51 (111 min)</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr"/>
-      <c r="F6" s="15" t="inlineStr"/>
+      <c r="E6" s="19" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -4285,198 +3503,166 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>25/03/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr"/>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr"/>
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Creation de la page principal</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Développement de la page principale (Home) incluant la structure globale et l'intégration du menu de navigation.</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(Home): Creation de la page principal  - Page principale - Menu de navigation</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr"/>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr"/>
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Créeation du journal de travail</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Mise en place opérationnelle du script Get_commit.sh et initialisation du document de suivi du journal de travail.</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>[3]</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Documentation(JNR): Créeation du journal de travail  mise en place du scripte Get_commit.sh</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr"/>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr"/>
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Featch interface</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Implémentation des appels interface (fetch) pour l'intégration et l'affichage dynamique de la liste des livres sur la page d'accueil.</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>[55]</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(interface): Featch interface  Affichage des livre sur la home page</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr"/>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr"/>
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Featch interface</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Correction et optimisation du script Get_commit.sh pour assurer la récupération des commits de la branche principale (main) et l'export correct des tâches dans le fichier CSV.</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>[20]</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Correction(Get_Commit): Correction du script Get_commit.sh pour récupérer les commits de la branche main et aussi les tache écrit dans le csv</t>
-        </is>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr"/>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr"/>
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>color menu</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Correction cosmétique et application de la charte graphique (couleurs) sur le menu de navigation.</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>[10]</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>Correction(shell): color menu</t>
-        </is>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr"/>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr"/>
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Save code on cloud</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Sauvegarde de sécurité de l'environnement de développement et externalisation du code source sur le cloud.</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>[7]</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>Tâche(Save): Save code on cloud</t>
-        </is>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr"/>
-      <c r="B15" s="15" t="inlineStr"/>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr"/>
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>2h15 (135 min)</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr"/>
-      <c r="F15" s="15" t="inlineStr"/>
+      <c r="E15" s="19" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -4484,222 +3670,185 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>01/04/2026</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr"/>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr"/>
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>ca ne fonctionnais pas chez mes camarades</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Résolution d'un problème d'exécution du script chez les autres collaborateurs suite à des modifications manuelles et non conformes des formats de dates.</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>[10]</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>il avait modif les dates et il ne faut surtout pas</t>
-        </is>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr"/>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr"/>
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Reload infini</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Identification et correction d'un anomalie provoquant une boucle de rechargement infinie (infinite reload) sur l'interface.</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>[6]</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
-        <is>
-          <t>Correction(Reload): Reload infini</t>
-        </is>
-      </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr"/>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr"/>
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>affiche les detail d'un livre avec le bouton pour lire</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Développement de la vue détaillée d'un ouvrage et intégration du bouton d'action pour lancer la lecture.</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>[15]</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(detail): affiche les detail d'un livre avec le bouton pour lire</t>
-        </is>
-      </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr"/>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr"/>
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Ouvre le pdf de résumer</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Implémentation de la fonctionnalité permettant l'ouverture et la consultation du résumé du livre au format PDF.</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(Résumé): Ouvre le pdf de résumer</t>
-        </is>
-      </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr"/>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr"/>
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>ajout d'un dark mode</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Début de l'intégration et configuration des styles pour le support du mode sombre (Dark Mode).</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>[20]</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>[WIP]</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(DarkMode): ajout d'un dark mode</t>
-        </is>
-      </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr"/>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr"/>
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>ouvire un epub</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Recherche et développement initial pour l'implémentation d'un lecteur de fichiers au format EPUB.</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>[WIP]</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(EPUB): ouvire un epub</t>
-        </is>
-      </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr"/>
-      <c r="B24" s="14" t="inlineStr"/>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Documentation(JNR)</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr"/>
+      <c r="B24" s="18" t="inlineStr"/>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Mise à jour régulière de la documentation du journal de travail.</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>[0]</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Documentation(JNR)</t>
-        </is>
-      </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr"/>
-      <c r="B25" s="15" t="inlineStr"/>
-      <c r="C25" s="16" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr"/>
+      <c r="B25" s="19" t="inlineStr"/>
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>2h11 (131 min)</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr"/>
-      <c r="F25" s="15" t="inlineStr"/>
+      <c r="E25" s="19" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
@@ -4707,86 +3856,74 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>22/04/2026</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr"/>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr"/>
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>interface de Théo</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Intégration et phase de tests avec la nouvelle interface fournie par Théo. Le serveur démarre correctement, mais des blocages persistent sur le traitement et le rendu des fichiers EPUB.</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>[1h30]</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(nouvelle interface): interface de Théo  Je n'arrive a pas grand chose pour le moment. ca run mais je n'arrive a rien avec les epub</t>
-        </is>
-      </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr"/>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr"/>
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>tentative de epub</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Nouvelles tentatives techniques pour parser et afficher le contenu des fichiers EPUB via l'interface, soucis de compatibilité en cours de résolution.</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>[1h30]</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>[WIP]</t>
         </is>
       </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(interface): tentative de epub  ca marche pas</t>
-        </is>
-      </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="15" t="inlineStr"/>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr"/>
+      <c r="B30" s="19" t="inlineStr"/>
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>3h00 (180 min)</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr"/>
-      <c r="F30" s="15" t="inlineStr"/>
+      <c r="E30" s="19" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
@@ -4794,86 +3931,74 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>29/04/2026</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr"/>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr"/>
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>lazy loading + interface improvements</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>Mise en place du chargement différé (lazy loading) pour optimiser les performances et améliorations globales de l'interface utilisateur (interface).</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Correction(loading): lazy loading + interface improvements</t>
-        </is>
-      </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr"/>
-      <c r="B34" s="17" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr"/>
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>interface custom</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Développement et ajustement d'endpoints spécifiques sur l'interface sur mesure (custom interface).</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>[10]</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité(interface): interface custom</t>
-        </is>
-      </c>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr"/>
-      <c r="B35" s="15" t="inlineStr"/>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr"/>
+      <c r="B35" s="19" t="inlineStr"/>
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>0h50 (50 min)</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr"/>
-      <c r="F35" s="15" t="inlineStr"/>
+      <c r="E35" s="19" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
@@ -4881,170 +4006,143 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>06/05/2026</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr"/>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr"/>
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>add custom interface for mobile</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>Adaptation et déploiement de l'interface personnalisée pour optimiser les requêtes provenant de l'application mobile.</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité: add custom interface for mobile</t>
-        </is>
-      </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr"/>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr"/>
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>add more champ de saisie on add page</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>Ajout de nouveaux champs de saisie (inputs) sur le formulaire de la page d'ajout pour enrichir les métadonnées.</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>[13]</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité: add more champ de saisie on add page</t>
-        </is>
-      </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr"/>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr"/>
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>sqlight</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>Configuration et intégration d'une base de données locale SQLite pour la persistance des données de l'application.</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
         <is>
           <t>[60]</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité: sqlight</t>
-        </is>
-      </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr"/>
-      <c r="B41" s="17" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr"/>
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>epub</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>Finalisation et validation fonctionnelle du module de lecture des fichiers EPUB.</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>[7]</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F41" s="13" t="inlineStr">
-        <is>
-          <t>Fonctionnalité: epub</t>
-        </is>
-      </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr"/>
-      <c r="B42" s="20" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr"/>
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>mise à jour journal de travail</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>Mise à jour des journal et maintenance du journal de suivi de projet.</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
-        <is>
-          <t>Tâche: mise à jour journal de travail</t>
-        </is>
-      </c>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="inlineStr"/>
-      <c r="B43" s="15" t="inlineStr"/>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr"/>
+      <c r="B43" s="19" t="inlineStr"/>
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D43" s="20" t="inlineStr">
         <is>
           <t>2h00 (120 min)</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr"/>
-      <c r="F43" s="15" t="inlineStr"/>
+      <c r="E43" s="19" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
@@ -5052,269 +4150,261 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>13/05/2026</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr"/>
-      <c r="B46" s="19" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr"/>
+      <c r="B46" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>JRN</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>Résolution d'un problème d'encodage et d'ouverture du fichier CSV sous Excel. Implémentation de la conversion automatisée au format XLSX pour garantir la compatibilité.</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>[40]</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F46" s="13" t="inlineStr">
-        <is>
-          <t>excel ne voulait pas ouvrir le csv alors j'ai du le convertir en xlsx et maintenant ça marche</t>
-        </is>
-      </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr"/>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr"/>
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>gestion erreurs reseau</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Amélioration de l'expérience utilisateur par l'ajout de messages d'erreur explicites en cas de perte de connexion ou d'inaccessibilité de l'interface.</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>[25]</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F47" s="13" t="inlineStr">
-        <is>
-          <t>ajout de messages d'erreur plus clairs quand l'interface est inaccessible</t>
-        </is>
-      </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr"/>
-      <c r="B48" s="17" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr"/>
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>url interface modifiable</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Ajout d'une option dans les paramètres de l'application permettant de modifier dynamiquement l'URL de base du serveur.</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>[30]</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E48" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F48" s="13" t="inlineStr">
-        <is>
-          <t>ajout d'un champ pour configurer l'url du serveur dans les parametres</t>
-        </is>
-      </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr"/>
-      <c r="B49" s="19" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr"/>
+      <c r="B49" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>detection emulateur vs telephone</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Développement d'une logique de détection réseau pour basculer automatiquement l'URL de l'interface entre localhost (émulateur Android) et l'adresse IP de la machine (smartphone physique).</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>[20]</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E49" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F49" s="13" t="inlineStr">
-        <is>
-          <t>correction de l'url par defaut selon le type d'appareil android</t>
-        </is>
-      </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr"/>
-      <c r="B50" s="23" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr"/>
+      <c r="B50" s="25" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>verification adb reverse</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>Tests de communication locale et validation du reverse-proxying à l'aide de la commande adb reverse tcp:3000 tcp:3000.</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>[15]</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E50" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F50" s="13" t="inlineStr">
-        <is>
-          <t>tests de connexion avec adb reverse tcp:3000 tcp:3000</t>
-        </is>
-      </c>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr"/>
-      <c r="B51" s="19" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr"/>
+      <c r="B51" s="23" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>interface / setings</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>Refactoring des appels de l'interface pour consommer dynamiquement l'URL configurée par l'utilisateur dans l'écran des paramètres.</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
         <is>
           <t>[10]</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E51" s="17" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="F51" s="13" t="inlineStr">
-        <is>
-          <t>call interface avec l'url configuré dans les settings</t>
-        </is>
-      </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr"/>
-      <c r="B52" s="20" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr"/>
+      <c r="B52" s="24" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>mise à jour journal de travail</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Génération et contrôle de la conformité du journal de travail.</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
+      <c r="E52" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="F52" s="13" t="inlineStr">
-        <is>
-          <t>Tâche: mise à jour journal de travail</t>
-        </is>
-      </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr"/>
-      <c r="B53" s="20" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr"/>
+      <c r="B53" s="19" t="inlineStr"/>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>2h20 (140 min)</t>
+        </is>
+      </c>
+      <c r="E53" s="19" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr"/>
+      <c r="B56" s="24" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>mise à jour journal de travail</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E56" s="17" t="inlineStr">
         <is>
           <t>[?]</t>
         </is>
       </c>
-      <c r="F53" s="13" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="15" t="inlineStr"/>
-      <c r="B54" s="15" t="inlineStr"/>
-      <c r="C54" s="16" t="inlineStr">
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr"/>
+      <c r="B57" s="19" t="inlineStr"/>
+      <c r="C57" s="20" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>2h20 (140 min)</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr"/>
-      <c r="F54" s="15" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>0h00 (0 min)</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
-  <mergeCells count="7">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A17:F17"/>
+  <autoFilter ref="A1:E58"/>
+  <mergeCells count="9">
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5326,52 +4416,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="11" min="1" max="1"/>
-    <col width="13" customWidth="1" style="11" min="2" max="2"/>
-    <col width="11" customWidth="1" style="11" min="3" max="3"/>
-    <col width="15" customWidth="1" style="11" min="4" max="4"/>
+    <col width="12" customWidth="1" style="15" min="1" max="1"/>
+    <col width="13" customWidth="1" style="15" min="2" max="2"/>
+    <col width="11" customWidth="1" style="15" min="3" max="3"/>
+    <col width="15" customWidth="1" style="15" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Total (min)</t>
         </is>
       </c>
-      <c r="C1" s="21" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>Total (h)</t>
         </is>
       </c>
-      <c r="D1" s="21" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>Total (h:min)</t>
         </is>
       </c>
-      <c r="F1" s="21" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="G1" s="21" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="I1" s="22" t="inlineStr">
+      <c r="I1" s="27" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="J1" s="22" t="inlineStr">
+      <c r="J1" s="27" t="inlineStr">
         <is>
           <t>Cumul (h)</t>
         </is>
@@ -5394,13 +4484,13 @@
           <t>1h51</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>Jours suivis</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -5428,7 +4518,7 @@
           <t>2h15</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="F3" s="27" t="inlineStr">
         <is>
           <t>Temps total</t>
         </is>
@@ -5464,14 +4554,14 @@
           <t>2h11</t>
         </is>
       </c>
-      <c r="F4" s="22" t="inlineStr">
+      <c r="F4" s="27" t="inlineStr">
         <is>
           <t>Moyenne / jour</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h04</t>
+          <t>1h48</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5500,7 +4590,7 @@
           <t>3h00</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="F5" s="27" t="inlineStr">
         <is>
           <t>Jour le plus chargé</t>
         </is>
@@ -5597,8 +4687,34 @@
         <v>14.45</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0h00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>14.45</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>